<commit_message>
Fixed parameters file instructions, added ignore to junk files
</commit_message>
<xml_diff>
--- a/Docker/parameters.xlsx
+++ b/Docker/parameters.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickbard/Desktop/CBG/BIP/Docker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{408EF992-34D0-E74D-B038-74857B4A8250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D08545D-DEA3-C943-BDA9-5D7D1A71312F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27860" yWindow="11460" windowWidth="28860" windowHeight="15700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="UMIs and Primers" sheetId="2" r:id="rId2"/>
     <sheet name="Dictionary Update" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2004" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2004" uniqueCount="465">
   <si>
     <t xml:space="preserve">NOTE: Parameters in red are mandatory </t>
   </si>
@@ -1396,9 +1396,6 @@
     <t>Max amplicon length</t>
   </si>
   <si>
-    <t>BOLDistilled_COI_Apr2026</t>
-  </si>
-  <si>
     <r>
       <t>BIP PARAMETERS FILE</t>
     </r>
@@ -1458,9 +1455,6 @@
     <t>Target Amplicon Length</t>
   </si>
   <si>
-    <t>BIN assign probability threshold</t>
-  </si>
-  <si>
     <t>e.g., 0.95</t>
   </si>
   <si>
@@ -1468,6 +1462,9 @@
   </si>
   <si>
     <t>e.g., 0.6</t>
+  </si>
+  <si>
+    <t>BOLDistilled_COI_</t>
   </si>
 </sst>
 </file>
@@ -2161,7 +2158,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2175,7 +2172,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -2231,7 +2228,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2240,7 +2237,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2249,7 +2246,7 @@
         <v>442</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2258,7 +2255,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2267,21 +2264,21 @@
         <v>26</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="6" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B16" s="22"/>
       <c r="C16" s="22"/>
@@ -2292,7 +2289,7 @@
         <v>23</v>
       </c>
       <c r="C17" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -2301,7 +2298,7 @@
         <v>24</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -2343,7 +2340,7 @@
     <row r="23" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="25"/>
       <c r="B23" s="26" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>17</v>
@@ -2352,7 +2349,7 @@
     <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="25"/>
       <c r="B24" s="26" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C24" s="24" t="s">
         <v>18</v>
@@ -2361,7 +2358,7 @@
     <row r="25" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="25"/>
       <c r="B25" s="26" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C25" s="24" t="s">
         <v>20</v>
@@ -2373,7 +2370,7 @@
         <v>233</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" x14ac:dyDescent="0.2">
@@ -2382,7 +2379,7 @@
         <v>234</v>
       </c>
       <c r="C27" s="24" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" x14ac:dyDescent="0.2">
@@ -2391,16 +2388,16 @@
         <v>235</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="25"/>
       <c r="B29" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="C29" s="24" t="s">
         <v>462</v>
-      </c>
-      <c r="C29" s="24" t="s">
-        <v>464</v>
       </c>
     </row>
   </sheetData>
@@ -8712,7 +8709,7 @@
         <v>239</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>446</v>
+        <v>464</v>
       </c>
       <c r="G2" s="18">
         <v>550</v>

</xml_diff>